<commit_message>
Fix: Preserve Excel rich text formatting for metadata and use native numbers in cell values
</commit_message>
<xml_diff>
--- a/scratch/test_output.xlsx
+++ b/scratch/test_output.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="96">
   <si>
     <r>
       <rPr>
@@ -463,6 +463,63 @@
   </si>
   <si>
     <t>Chirag Nayak</t>
+  </si>
+  <si>
+    <t>TEST_ID</t>
+  </si>
+  <si>
+    <t>STUDENT NAME</t>
+  </si>
+  <si>
+    <t>CAMPUS</t>
+  </si>
+  <si>
+    <t>0.8</t>
+  </si>
+  <si>
+    <t>0.9</t>
+  </si>
+  <si>
+    <t>TEST_ID_2</t>
+  </si>
+  <si>
+    <t>STUDENT NAME 2</t>
+  </si>
+  <si>
+    <t>CAMPUS 2</t>
+  </si>
+  <si>
+    <t>0.79</t>
+  </si>
+  <si>
+    <t>0.85</t>
+  </si>
+  <si>
+    <t>0.78</t>
+  </si>
+  <si>
+    <t>0.77</t>
+  </si>
+  <si>
+    <t>Niranjan gowda .</t>
+  </si>
+  <si>
+    <t>CHINMAY ASHWA K</t>
+  </si>
+  <si>
+    <t>Shriya M Bhat</t>
+  </si>
+  <si>
+    <t>DIVYESH R</t>
+  </si>
+  <si>
+    <t>Samarth S .</t>
+  </si>
+  <si>
+    <t>Kirti Kumar</t>
+  </si>
+  <si>
+    <t>VEERESH N M .</t>
   </si>
   <si>
     <t>Sridhar Gowda s</t>
@@ -1684,21 +1741,435 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="39">
+        <v>250</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="41">
+        <v>1</v>
+      </c>
+      <c r="G12" s="39">
+        <v>90</v>
+      </c>
+      <c r="H12" s="41">
+        <v>2</v>
+      </c>
+      <c r="I12" s="40" t="s">
+        <v>29</v>
+      </c>
+      <c r="J12" s="39">
+        <v>80</v>
+      </c>
+      <c r="K12" s="41">
+        <v>3</v>
+      </c>
+      <c r="L12" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="M12" s="39">
+        <v>80</v>
+      </c>
+      <c r="N12" s="41">
+        <v>4</v>
+      </c>
+      <c r="O12" s="40" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="39">
+        <v>240</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="41">
+        <v>2</v>
+      </c>
+      <c r="G13" s="39">
+        <v>85</v>
+      </c>
+      <c r="H13" s="41">
+        <v>3</v>
+      </c>
+      <c r="I13" s="40" t="s">
+        <v>34</v>
+      </c>
+      <c r="J13" s="39">
+        <v>78</v>
+      </c>
+      <c r="K13" s="41">
+        <v>4</v>
+      </c>
+      <c r="L13" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="M13" s="39">
+        <v>77</v>
+      </c>
+      <c r="N13" s="41">
+        <v>5</v>
+      </c>
+      <c r="O13" s="40" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="36">
+        <v>268405555</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="39">
+        <v>72</v>
+      </c>
+      <c r="E14" s="40">
+        <v>24</v>
+      </c>
+      <c r="F14" s="41">
+        <v>438</v>
+      </c>
+      <c r="G14" s="39">
+        <v>23</v>
+      </c>
+      <c r="H14" s="41">
+        <v>662</v>
+      </c>
+      <c r="I14" s="40">
+        <v>23</v>
+      </c>
+      <c r="J14" s="39">
+        <v>30</v>
+      </c>
+      <c r="K14" s="41">
+        <v>184</v>
+      </c>
+      <c r="L14" s="40">
+        <v>30</v>
+      </c>
+      <c r="M14" s="39">
+        <v>19</v>
+      </c>
+      <c r="N14" s="41">
+        <v>880</v>
+      </c>
+      <c r="O14" s="40">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="36">
+        <v>235417136</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="39">
+        <v>69</v>
+      </c>
+      <c r="E15" s="40">
+        <v>23</v>
+      </c>
+      <c r="F15" s="41">
+        <v>474</v>
+      </c>
+      <c r="G15" s="39">
+        <v>36</v>
+      </c>
+      <c r="H15" s="41">
+        <v>262</v>
+      </c>
+      <c r="I15" s="40">
+        <v>36</v>
+      </c>
+      <c r="J15" s="39">
+        <v>19</v>
+      </c>
+      <c r="K15" s="41">
+        <v>497</v>
+      </c>
+      <c r="L15" s="40">
+        <v>19</v>
+      </c>
+      <c r="M15" s="39">
+        <v>14</v>
+      </c>
+      <c r="N15" s="41">
+        <v>1178</v>
+      </c>
+      <c r="O15" s="40">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="36">
+        <v>235417064</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="39">
+        <v>69</v>
+      </c>
+      <c r="E16" s="40">
+        <v>23</v>
+      </c>
+      <c r="F16" s="41">
+        <v>475</v>
+      </c>
+      <c r="G16" s="39">
+        <v>35</v>
+      </c>
+      <c r="H16" s="41">
+        <v>281</v>
+      </c>
+      <c r="I16" s="40">
+        <v>35</v>
+      </c>
+      <c r="J16" s="39">
+        <v>19</v>
+      </c>
+      <c r="K16" s="41">
+        <v>497</v>
+      </c>
+      <c r="L16" s="40">
+        <v>19</v>
+      </c>
+      <c r="M16" s="39">
+        <v>15</v>
+      </c>
+      <c r="N16" s="41">
+        <v>1110</v>
+      </c>
+      <c r="O16" s="40">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="36">
+        <v>235417465</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="39">
+        <v>66</v>
+      </c>
+      <c r="E17" s="40">
+        <v>22</v>
+      </c>
+      <c r="F17" s="41">
+        <v>514</v>
+      </c>
+      <c r="G17" s="39">
+        <v>36</v>
+      </c>
+      <c r="H17" s="41">
+        <v>262</v>
+      </c>
+      <c r="I17" s="40">
+        <v>36</v>
+      </c>
+      <c r="J17" s="39">
+        <v>16</v>
+      </c>
+      <c r="K17" s="41">
+        <v>661</v>
+      </c>
+      <c r="L17" s="40">
+        <v>16</v>
+      </c>
+      <c r="M17" s="39">
+        <v>14</v>
+      </c>
+      <c r="N17" s="41">
+        <v>1178</v>
+      </c>
+      <c r="O17" s="40">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="36">
+        <v>268427244</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="39">
+        <v>62</v>
+      </c>
+      <c r="E18" s="40">
+        <v>20.67</v>
+      </c>
+      <c r="F18" s="41">
+        <v>591</v>
+      </c>
+      <c r="G18" s="39">
+        <v>37</v>
+      </c>
+      <c r="H18" s="41">
+        <v>237</v>
+      </c>
+      <c r="I18" s="40">
+        <v>37</v>
+      </c>
+      <c r="J18" s="39">
+        <v>14</v>
+      </c>
+      <c r="K18" s="41">
+        <v>838</v>
+      </c>
+      <c r="L18" s="40">
+        <v>14</v>
+      </c>
+      <c r="M18" s="39">
+        <v>11</v>
+      </c>
+      <c r="N18" s="41">
+        <v>1379</v>
+      </c>
+      <c r="O18" s="40">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="36">
+        <v>246411627</v>
+      </c>
+      <c r="B19" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="39">
+        <v>58</v>
+      </c>
+      <c r="E19" s="40">
+        <v>19.33</v>
+      </c>
+      <c r="F19" s="41">
+        <v>686</v>
+      </c>
+      <c r="G19" s="39">
+        <v>21</v>
+      </c>
+      <c r="H19" s="41">
+        <v>762</v>
+      </c>
+      <c r="I19" s="40">
+        <v>21</v>
+      </c>
+      <c r="J19" s="39">
+        <v>26</v>
+      </c>
+      <c r="K19" s="41">
+        <v>251</v>
+      </c>
+      <c r="L19" s="40">
+        <v>26</v>
+      </c>
+      <c r="M19" s="39">
+        <v>11</v>
+      </c>
+      <c r="N19" s="41">
+        <v>1379</v>
+      </c>
+      <c r="O19" s="40">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="36">
+        <v>268428290</v>
+      </c>
+      <c r="B20" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="39">
+        <v>58</v>
+      </c>
+      <c r="E20" s="40">
+        <v>19.33</v>
+      </c>
+      <c r="F20" s="41">
+        <v>687</v>
+      </c>
+      <c r="G20" s="39">
+        <v>20</v>
+      </c>
+      <c r="H20" s="41">
+        <v>813</v>
+      </c>
+      <c r="I20" s="40">
+        <v>20</v>
+      </c>
+      <c r="J20" s="39">
+        <v>7</v>
+      </c>
+      <c r="K20" s="41">
+        <v>1482</v>
+      </c>
+      <c r="L20" s="40">
+        <v>7</v>
+      </c>
+      <c r="M20" s="39">
+        <v>31</v>
+      </c>
+      <c r="N20" s="41">
+        <v>418</v>
+      </c>
+      <c r="O20" s="40">
+        <v>31</v>
+      </c>
+    </row>
     <row r="21" ht="18" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="36">
         <v>257396742</v>
       </c>
       <c r="B21" s="37" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C21" s="38" t="s">
         <v>23</v>
@@ -1745,7 +2216,7 @@
         <v>235417327</v>
       </c>
       <c r="B22" s="37" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="C22" s="38" t="s">
         <v>23</v>
@@ -1792,7 +2263,7 @@
         <v>235417122</v>
       </c>
       <c r="B23" s="37" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="C23" s="38" t="s">
         <v>23</v>
@@ -1839,7 +2310,7 @@
         <v>268406003</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="C24" s="38" t="s">
         <v>23</v>
@@ -1886,7 +2357,7 @@
         <v>268404990</v>
       </c>
       <c r="B25" s="37" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>23</v>
@@ -1933,7 +2404,7 @@
         <v>268401754</v>
       </c>
       <c r="B26" s="37" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="C26" s="38" t="s">
         <v>23</v>
@@ -1980,7 +2451,7 @@
         <v>268410670</v>
       </c>
       <c r="B27" s="37" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="C27" s="38" t="s">
         <v>23</v>
@@ -2027,7 +2498,7 @@
         <v>268423534</v>
       </c>
       <c r="B28" s="37" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="C28" s="38" t="s">
         <v>23</v>
@@ -2074,7 +2545,7 @@
         <v>268411723</v>
       </c>
       <c r="B29" s="37" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C29" s="38" t="s">
         <v>23</v>
@@ -2121,7 +2592,7 @@
         <v>235417482</v>
       </c>
       <c r="B30" s="37" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="C30" s="38" t="s">
         <v>23</v>
@@ -2168,7 +2639,7 @@
         <v>246415117</v>
       </c>
       <c r="B31" s="37" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="C31" s="38" t="s">
         <v>23</v>
@@ -2215,7 +2686,7 @@
         <v>268410102</v>
       </c>
       <c r="B32" s="37" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="C32" s="38" t="s">
         <v>23</v>
@@ -2262,7 +2733,7 @@
         <v>268401852</v>
       </c>
       <c r="B33" s="37" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="C33" s="38" t="s">
         <v>23</v>
@@ -2309,7 +2780,7 @@
         <v>268407948</v>
       </c>
       <c r="B34" s="37" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="C34" s="38" t="s">
         <v>23</v>
@@ -2356,7 +2827,7 @@
         <v>246549501</v>
       </c>
       <c r="B35" s="37" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="C35" s="38" t="s">
         <v>23</v>
@@ -2403,7 +2874,7 @@
         <v>268410973</v>
       </c>
       <c r="B36" s="37" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="C36" s="38" t="s">
         <v>23</v>
@@ -2450,7 +2921,7 @@
         <v>268401372</v>
       </c>
       <c r="B37" s="37" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="C37" s="38" t="s">
         <v>23</v>
@@ -2497,7 +2968,7 @@
         <v>268410002</v>
       </c>
       <c r="B38" s="37" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C38" s="38" t="s">
         <v>23</v>
@@ -2544,7 +3015,7 @@
         <v>268404100</v>
       </c>
       <c r="B39" s="37" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="C39" s="38" t="s">
         <v>23</v>
@@ -2591,7 +3062,7 @@
         <v>268401716</v>
       </c>
       <c r="B40" s="37" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C40" s="38" t="s">
         <v>23</v>
@@ -2638,7 +3109,7 @@
         <v>268404104</v>
       </c>
       <c r="B41" s="37" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="C41" s="38" t="s">
         <v>23</v>
@@ -2685,7 +3156,7 @@
         <v>235418218</v>
       </c>
       <c r="B42" s="37" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="C42" s="38" t="s">
         <v>23</v>
@@ -2732,7 +3203,7 @@
         <v>235417499</v>
       </c>
       <c r="B43" s="37" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="C43" s="38" t="s">
         <v>23</v>
@@ -2779,7 +3250,7 @@
         <v>268424269</v>
       </c>
       <c r="B44" s="37" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="C44" s="38" t="s">
         <v>23</v>
@@ -2826,7 +3297,7 @@
         <v>268409964</v>
       </c>
       <c r="B45" s="37" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="C45" s="38" t="s">
         <v>23</v>
@@ -2873,7 +3344,7 @@
         <v>268404737</v>
       </c>
       <c r="B46" s="37" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="C46" s="38" t="s">
         <v>23</v>
@@ -2920,7 +3391,7 @@
         <v>268400126</v>
       </c>
       <c r="B47" s="37" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="C47" s="38" t="s">
         <v>23</v>
@@ -2967,7 +3438,7 @@
         <v>268401906</v>
       </c>
       <c r="B48" s="37" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C48" s="38" t="s">
         <v>23</v>
@@ -3014,7 +3485,7 @@
         <v>268408437</v>
       </c>
       <c r="B49" s="37" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="C49" s="38" t="s">
         <v>23</v>
@@ -3061,7 +3532,7 @@
         <v>246415119</v>
       </c>
       <c r="B50" s="37" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="C50" s="38" t="s">
         <v>23</v>
@@ -3108,7 +3579,7 @@
         <v>268404255</v>
       </c>
       <c r="B51" s="37" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="C51" s="38" t="s">
         <v>23</v>
@@ -3155,7 +3626,7 @@
         <v>268406744</v>
       </c>
       <c r="B52" s="37" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="C52" s="38" t="s">
         <v>23</v>
@@ -3202,7 +3673,7 @@
         <v>268405683</v>
       </c>
       <c r="B53" s="37" t="s">
-        <v>57</v>
+        <v>76</v>
       </c>
       <c r="C53" s="38" t="s">
         <v>23</v>
@@ -3249,7 +3720,7 @@
         <v>235417017</v>
       </c>
       <c r="B54" s="37" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="C54" s="38" t="s">
         <v>23</v>
@@ -3296,7 +3767,7 @@
         <v>235419636</v>
       </c>
       <c r="B55" s="37" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C55" s="38" t="s">
         <v>23</v>
@@ -3343,7 +3814,7 @@
         <v>268410955</v>
       </c>
       <c r="B56" s="37" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="C56" s="38" t="s">
         <v>23</v>
@@ -3390,7 +3861,7 @@
         <v>268404453</v>
       </c>
       <c r="B57" s="37" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="C57" s="38" t="s">
         <v>23</v>
@@ -3437,7 +3908,7 @@
         <v>268404742</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="C58" s="38" t="s">
         <v>23</v>
@@ -3484,7 +3955,7 @@
         <v>268400778</v>
       </c>
       <c r="B59" s="37" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="C59" s="38" t="s">
         <v>23</v>
@@ -3531,7 +4002,7 @@
         <v>235418311</v>
       </c>
       <c r="B60" s="37" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="C60" s="38" t="s">
         <v>23</v>
@@ -3578,7 +4049,7 @@
         <v>268405156</v>
       </c>
       <c r="B61" s="37" t="s">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="C61" s="38" t="s">
         <v>23</v>
@@ -3625,7 +4096,7 @@
         <v>235418115</v>
       </c>
       <c r="B62" s="37" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="C62" s="38" t="s">
         <v>23</v>
@@ -3672,7 +4143,7 @@
         <v>268404905</v>
       </c>
       <c r="B63" s="37" t="s">
-        <v>67</v>
+        <v>86</v>
       </c>
       <c r="C63" s="38" t="s">
         <v>23</v>
@@ -3719,7 +4190,7 @@
         <v>268402246</v>
       </c>
       <c r="B64" s="37" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="C64" s="38" t="s">
         <v>23</v>
@@ -3766,7 +4237,7 @@
         <v>268403476</v>
       </c>
       <c r="B65" s="37" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="C65" s="38" t="s">
         <v>23</v>
@@ -3813,7 +4284,7 @@
         <v>268404541</v>
       </c>
       <c r="B66" s="37" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="C66" s="38" t="s">
         <v>23</v>
@@ -3860,7 +4331,7 @@
         <v>268407105</v>
       </c>
       <c r="B67" s="37" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="C67" s="38" t="s">
         <v>23</v>
@@ -3907,7 +4378,7 @@
         <v>268406245</v>
       </c>
       <c r="B68" s="37" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="C68" s="38" t="s">
         <v>23</v>
@@ -3954,7 +4425,7 @@
         <v>268401663</v>
       </c>
       <c r="B69" s="37" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="C69" s="38" t="s">
         <v>23</v>
@@ -4001,7 +4472,7 @@
         <v>235419637</v>
       </c>
       <c r="B70" s="37" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="C70" s="38" t="s">
         <v>23</v>
@@ -4048,7 +4519,7 @@
         <v>246415123</v>
       </c>
       <c r="B71" s="37" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="C71" s="38" t="s">
         <v>23</v>
@@ -4095,7 +4566,7 @@
         <v>268411070</v>
       </c>
       <c r="B72" s="37" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="C72" s="38" t="s">
         <v>23</v>

</xml_diff>